<commit_message>
Add plot checks, per-lesson languages and three beginner lessons
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw_export.xlsx
+++ b/data/raw_export.xlsx
@@ -679,10 +679,10 @@
     <t xml:space="preserve">R_0045</t>
   </si>
   <si>
-    <t xml:space="preserve">3/12/2026 10:22 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/12/2026 10:27 </t>
+    <t xml:space="preserve">3/12/2026 10:22 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/12/2026 10:27 PM</t>
   </si>
   <si>
     <t xml:space="preserve">20 years</t>
@@ -694,7 +694,7 @@
     <t xml:space="preserve">13.03.2026 04:54</t>
   </si>
   <si>
-    <t xml:space="preserve">3/13/2026 05:02 </t>
+    <t xml:space="preserve">3/13/2026 05:02 AM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0047</t>
@@ -703,7 +703,7 @@
     <t xml:space="preserve">13.03.2026 15:25</t>
   </si>
   <si>
-    <t xml:space="preserve">3/13/2026 03:30 </t>
+    <t xml:space="preserve">3/13/2026 03:30 PM</t>
   </si>
   <si>
     <t xml:space="preserve">28</t>
@@ -715,7 +715,7 @@
     <t xml:space="preserve">13.03.2026 16:50</t>
   </si>
   <si>
-    <t xml:space="preserve">3/13/2026 04:57 </t>
+    <t xml:space="preserve">3/13/2026 04:57 PM</t>
   </si>
   <si>
     <t xml:space="preserve">26</t>
@@ -733,10 +733,10 @@
     <t xml:space="preserve">R_0050</t>
   </si>
   <si>
-    <t xml:space="preserve">3/14/2026 12:58 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/14/2026 01:11 </t>
+    <t xml:space="preserve">3/14/2026 12:58 AM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/14/2026 01:11 AM</t>
   </si>
   <si>
     <t xml:space="preserve">51</t>
@@ -745,7 +745,7 @@
     <t xml:space="preserve">R_0051</t>
   </si>
   <si>
-    <t xml:space="preserve">3/14/2026 05:19 </t>
+    <t xml:space="preserve">3/14/2026 05:19 PM</t>
   </si>
   <si>
     <t xml:space="preserve">14.03.2026 17:26</t>
@@ -778,10 +778,10 @@
     <t xml:space="preserve">R_0054</t>
   </si>
   <si>
-    <t xml:space="preserve">3/16/2026 07:28 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/16/2026 07:31 </t>
+    <t xml:space="preserve">3/16/2026 07:28 AM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/16/2026 07:31 AM</t>
   </si>
   <si>
     <t xml:space="preserve">52</t>
@@ -802,7 +802,7 @@
     <t xml:space="preserve">R_0056</t>
   </si>
   <si>
-    <t xml:space="preserve">3/16/2026 11:16 </t>
+    <t xml:space="preserve">3/16/2026 11:16 AM</t>
   </si>
   <si>
     <t xml:space="preserve">16.03.2026 11:21</t>
@@ -814,7 +814,7 @@
     <t xml:space="preserve">16.03.2026 23:46</t>
   </si>
   <si>
-    <t xml:space="preserve">3/16/2026 11:49 </t>
+    <t xml:space="preserve">3/16/2026 11:49 PM</t>
   </si>
   <si>
     <t xml:space="preserve">40</t>
@@ -823,7 +823,7 @@
     <t xml:space="preserve">R_0058</t>
   </si>
   <si>
-    <t xml:space="preserve">3/17/2026 02:55 </t>
+    <t xml:space="preserve">3/17/2026 02:55 AM</t>
   </si>
   <si>
     <t xml:space="preserve">17.03.2026 03:00</t>
@@ -835,22 +835,22 @@
     <t xml:space="preserve">17.03.2026 08:32</t>
   </si>
   <si>
-    <t xml:space="preserve">3/17/2026 08:36 </t>
+    <t xml:space="preserve">3/17/2026 08:36 AM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0060</t>
   </si>
   <si>
-    <t xml:space="preserve">3/17/2026 10:05 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/17/2026 10:08 </t>
+    <t xml:space="preserve">3/17/2026 10:05 AM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/17/2026 10:08 AM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0061</t>
   </si>
   <si>
-    <t xml:space="preserve">3/17/2026 02:43 </t>
+    <t xml:space="preserve">3/17/2026 02:43 PM</t>
   </si>
   <si>
     <t xml:space="preserve">17.03.2026 14:51</t>
@@ -865,13 +865,13 @@
     <t xml:space="preserve">17.03.2026 22:41</t>
   </si>
   <si>
-    <t xml:space="preserve">3/17/2026 10:46 </t>
+    <t xml:space="preserve">3/17/2026 10:46 PM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0063</t>
   </si>
   <si>
-    <t xml:space="preserve">3/18/2026 05:13 </t>
+    <t xml:space="preserve">3/18/2026 05:13 AM</t>
   </si>
   <si>
     <t xml:space="preserve">18.03.2026 05:18</t>
@@ -883,25 +883,25 @@
     <t xml:space="preserve">18.03.2026 07:22</t>
   </si>
   <si>
-    <t xml:space="preserve">3/18/2026 07:29 </t>
+    <t xml:space="preserve">3/18/2026 07:29 AM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0065</t>
   </si>
   <si>
-    <t xml:space="preserve">3/18/2026 10:35 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/18/2026 10:45 </t>
+    <t xml:space="preserve">3/18/2026 10:35 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/18/2026 10:45 PM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0066</t>
   </si>
   <si>
-    <t xml:space="preserve">3/19/2026 08:58 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/19/2026 09:08 </t>
+    <t xml:space="preserve">3/19/2026 08:58 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/19/2026 09:08 PM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0067</t>
@@ -919,10 +919,10 @@
     <t xml:space="preserve">R_0068</t>
   </si>
   <si>
-    <t xml:space="preserve">3/20/2026 08:18 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/20/2026 08:22 </t>
+    <t xml:space="preserve">3/20/2026 08:18 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/20/2026 08:22 PM</t>
   </si>
   <si>
     <t xml:space="preserve">57</t>
@@ -934,7 +934,7 @@
     <t xml:space="preserve">21.03.2026 03:05</t>
   </si>
   <si>
-    <t xml:space="preserve">3/21/2026 03:10 </t>
+    <t xml:space="preserve">3/21/2026 03:10 AM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0070</t>
@@ -949,7 +949,7 @@
     <t xml:space="preserve">R_0071</t>
   </si>
   <si>
-    <t xml:space="preserve">3/21/2026 07:08 </t>
+    <t xml:space="preserve">3/21/2026 07:08 AM</t>
   </si>
   <si>
     <t xml:space="preserve">21.03.2026 07:11</t>
@@ -961,34 +961,34 @@
     <t xml:space="preserve">21.03.2026 10:24</t>
   </si>
   <si>
-    <t xml:space="preserve">3/21/2026 10:27 </t>
+    <t xml:space="preserve">3/21/2026 10:27 AM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0073</t>
   </si>
   <si>
-    <t xml:space="preserve">3/21/2026 01:26 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/21/2026 01:36 </t>
+    <t xml:space="preserve">3/21/2026 01:26 PM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/21/2026 01:36 PM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0074</t>
   </si>
   <si>
-    <t xml:space="preserve">3/22/2026 07:54 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/22/2026 08:00 </t>
+    <t xml:space="preserve">3/22/2026 07:54 AM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/22/2026 08:00 AM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0075</t>
   </si>
   <si>
-    <t xml:space="preserve">3/22/2026 10:56 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3/22/2026 11:08 </t>
+    <t xml:space="preserve">3/22/2026 10:56 AM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3/22/2026 11:08 AM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0076</t>
@@ -997,13 +997,13 @@
     <t xml:space="preserve">22.03.2026 11:45</t>
   </si>
   <si>
-    <t xml:space="preserve">3/22/2026 11:51 </t>
+    <t xml:space="preserve">3/22/2026 11:51 AM</t>
   </si>
   <si>
     <t xml:space="preserve">R_0077</t>
   </si>
   <si>
-    <t xml:space="preserve">3/22/2026 04:43 </t>
+    <t xml:space="preserve">3/22/2026 04:43 PM</t>
   </si>
   <si>
     <t xml:space="preserve">22.03.2026 16:46</t>
@@ -1018,7 +1018,7 @@
     <t xml:space="preserve">23.03.2026 04:19</t>
   </si>
   <si>
-    <t xml:space="preserve">3/23/2026 04:25 </t>
+    <t xml:space="preserve">3/23/2026 04:25 AM</t>
   </si>
   <si>
     <t xml:space="preserve">Total responses: 82</t>

</xml_diff>